<commit_message>
#7 Added links for peripheral in word DOC and PDF
</commit_message>
<xml_diff>
--- a/Design Files/Oil-Diffuser-A-v1.0.0/BOM/Client-BOM-Oil-Diffuser-A-v1.0.0.xlsx
+++ b/Design Files/Oil-Diffuser-A-v1.0.0/BOM/Client-BOM-Oil-Diffuser-A-v1.0.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\elliotrosenberg-oildiffuser\Design Files\Oil-Diffuser-A-v1.0.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="211">
   <si>
     <t>#</t>
   </si>
@@ -642,29 +642,23 @@
     <t>24v 2 Amp US plug</t>
   </si>
   <si>
-    <t>AC 250V 6A On/Off Prewired Standard Toggle Switch With Wire Cable KNS-1 SPST Contacts Switch Electrical Equipment</t>
-  </si>
-  <si>
     <t>Toggle Switch</t>
   </si>
   <si>
-    <t>1Pcs Gdstime DC 24V 75mm x 30mm Centrifugal Blower Fan 7530 7.5cm Dual Ball Turbo Radiator Fan 75mm Purifier Heatsink Fan</t>
-  </si>
-  <si>
     <t>24V Sleeve XH2.54</t>
   </si>
   <si>
-    <t>D16mm 1.7MHz Ultrasonic Mist Maker Atomizing Transducer Ceramic Humidifier</t>
-  </si>
-  <si>
     <t>16mm 1.7MHz</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -724,8 +718,28 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color indexed="12"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color indexed="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -744,8 +758,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -836,11 +856,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -886,9 +920,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -898,8 +929,18 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1186,7 +1227,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
@@ -1200,7 +1241,7 @@
     <col min="11" max="11" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="15.75" thickBot="1">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1209,11 +1250,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1246,7 +1287,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="48.75" thickBot="1">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1278,7 +1319,7 @@
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="36.75" thickBot="1">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B38" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1310,7 +1351,7 @@
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="48.75" thickBot="1">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1342,7 +1383,7 @@
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15.75" thickBot="1">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1374,7 +1415,7 @@
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="24.75" thickBot="1">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1406,7 +1447,7 @@
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15.75" thickBot="1">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1438,7 +1479,7 @@
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="15.75" thickBot="1">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1470,7 +1511,7 @@
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="36.75" thickBot="1">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1502,7 +1543,7 @@
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15.75" thickBot="1">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1534,7 +1575,7 @@
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="24.75" thickBot="1">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1566,7 +1607,7 @@
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15.75" thickBot="1">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1598,7 +1639,7 @@
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="36.75" thickBot="1">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -1630,7 +1671,7 @@
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="48.75" thickBot="1">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1662,7 +1703,7 @@
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="48.75" thickBot="1">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -1671,32 +1712,32 @@
       <c r="C16" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="18" t="s">
         <v>71</v>
       </c>
       <c r="F16" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="18" t="s">
+      <c r="H16" s="17" t="s">
         <v>162</v>
       </c>
       <c r="I16" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="J16" s="18">
+      <c r="J16" s="17">
         <v>1</v>
       </c>
       <c r="K16" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="24.75" thickBot="1">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -1728,7 +1769,7 @@
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="24.75" thickBot="1">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1760,7 +1801,7 @@
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="24.75" thickBot="1">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1792,7 +1833,7 @@
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="36.75" thickBot="1">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -1824,7 +1865,7 @@
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="15.75" thickBot="1">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -1856,7 +1897,7 @@
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="36.75" thickBot="1">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -1888,7 +1929,7 @@
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="24.75" thickBot="1">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1920,7 +1961,7 @@
       </c>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15.75" thickBot="1">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -1952,7 +1993,7 @@
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="15.75" thickBot="1">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -1984,7 +2025,7 @@
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="36.75" thickBot="1">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -2016,7 +2057,7 @@
       </c>
       <c r="K26" s="9"/>
     </row>
-    <row r="27" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="24.75" thickBot="1">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -2050,7 +2091,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="15.75" thickBot="1">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -2082,7 +2123,7 @@
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="15.75" thickBot="1">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -2114,7 +2155,7 @@
       </c>
       <c r="K29" s="7"/>
     </row>
-    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="15.75" thickBot="1">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
@@ -2146,7 +2187,7 @@
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="36.75" thickBot="1">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
@@ -2178,7 +2219,7 @@
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="15.75" thickBot="1">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
@@ -2210,7 +2251,7 @@
       </c>
       <c r="K32" s="9"/>
     </row>
-    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="15.75" thickBot="1">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -2240,7 +2281,7 @@
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="15.75" thickBot="1">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
@@ -2272,7 +2313,7 @@
       </c>
       <c r="K34" s="9"/>
     </row>
-    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="15.75" thickBot="1">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f>ROW(B35) - ROW($B$2)</f>
@@ -2304,7 +2345,7 @@
       </c>
       <c r="K35" s="7"/>
     </row>
-    <row r="36" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="36.75" thickBot="1">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
         <f t="shared" si="0"/>
@@ -2336,7 +2377,7 @@
       </c>
       <c r="K36" s="9"/>
     </row>
-    <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="15.75" thickBot="1">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
         <f>ROW(B37) - ROW($B$2)</f>
@@ -2368,7 +2409,7 @@
       </c>
       <c r="K37" s="7"/>
     </row>
-    <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="15.75" thickBot="1">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
         <f t="shared" si="0"/>
@@ -2400,7 +2441,7 @@
       </c>
       <c r="K38" s="9"/>
     </row>
-    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="15.75" thickBot="1">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
         <f>ROW(B39) - ROW($B$2)</f>
@@ -2432,7 +2473,7 @@
       </c>
       <c r="K39" s="7"/>
     </row>
-    <row r="40" spans="1:11" ht="25.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="25.5" thickBot="1">
       <c r="B40" s="11">
         <f t="shared" ref="B40:B43" si="1">ROW(B40) - ROW($B$2)</f>
         <v>38</v>
@@ -2443,7 +2484,7 @@
       <c r="D40" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="E40" s="20" t="s">
+      <c r="E40" s="19" t="s">
         <v>205</v>
       </c>
       <c r="F40" s="7" t="s">
@@ -2461,9 +2502,11 @@
       <c r="J40" s="7">
         <v>1</v>
       </c>
-      <c r="K40" s="7"/>
-    </row>
-    <row r="41" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K40" s="21" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="15.75" thickBot="1">
       <c r="B41" s="11">
         <f t="shared" si="1"/>
         <v>39</v>
@@ -2474,14 +2517,14 @@
       <c r="D41" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="E41" s="7" t="s">
+      <c r="E41" s="22" t="s">
         <v>207</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>201</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H41" s="7" t="s">
         <v>201</v>
@@ -2492,9 +2535,11 @@
       <c r="J41" s="7">
         <v>1</v>
       </c>
-      <c r="K41" s="7"/>
-    </row>
-    <row r="42" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K41" s="21" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="15.75" thickBot="1">
       <c r="B42" s="11">
         <f t="shared" si="1"/>
         <v>40</v>
@@ -2505,27 +2550,29 @@
       <c r="D42" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="E42" s="7" t="s">
-        <v>209</v>
+      <c r="E42" s="22" t="s">
+        <v>208</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>201</v>
       </c>
       <c r="G42" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="I42" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="J42" s="7">
+        <v>1</v>
+      </c>
+      <c r="K42" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="H42" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="I42" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="J42" s="7">
-        <v>1</v>
-      </c>
-      <c r="K42" s="7"/>
-    </row>
-    <row r="43" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:11" ht="15.75" thickBot="1">
       <c r="B43" s="11">
         <f t="shared" si="1"/>
         <v>41</v>
@@ -2536,14 +2583,14 @@
       <c r="D43" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="E43" s="7" t="s">
-        <v>211</v>
+      <c r="E43" s="22" t="s">
+        <v>209</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>201</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H43" s="7" t="s">
         <v>201</v>
@@ -2554,13 +2601,21 @@
       <c r="J43" s="7">
         <v>1</v>
       </c>
-      <c r="K43" s="7"/>
+      <c r="K43" s="21" t="s">
+        <v>210</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K40" r:id="rId1"/>
+    <hyperlink ref="K41" r:id="rId2"/>
+    <hyperlink ref="K42" r:id="rId3"/>
+    <hyperlink ref="K43" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>